<commit_message>
perbaikan nama di index blade
</commit_message>
<xml_diff>
--- a/public/assets/file/Mini PC.xlsx
+++ b/public/assets/file/Mini PC.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="109">
   <si>
     <t>No</t>
   </si>
@@ -234,9 +234,6 @@
     <t>DHCP - Man. Casemix</t>
   </si>
   <si>
-    <t>CPU: Intel Core i3 - 7100U 2,4Ghz (4 CPUs)</t>
-  </si>
-  <si>
     <t>RAM: 4GB DDR 4</t>
   </si>
   <si>
@@ -337,6 +334,18 @@
   </si>
   <si>
     <t>192.168.121.137</t>
+  </si>
+  <si>
+    <t>CPU: Intel Core i3 - 7100U 2,4Ghz</t>
+  </si>
+  <si>
+    <t>CPU: Intel Core i3 - 10110U 2,1Ghz</t>
+  </si>
+  <si>
+    <t>CPU: Celeron J4025 - 2.00GHz</t>
+  </si>
+  <si>
+    <t>CPU: i5-1240P - 1.7GHz</t>
   </si>
 </sst>
 </file>
@@ -749,13 +758,13 @@
         <v>1</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G2" t="s">
-        <v>71</v>
+        <v>105</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -772,10 +781,13 @@
         <v>1</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
+      </c>
+      <c r="F3" t="s">
+        <v>71</v>
       </c>
       <c r="G3" t="s">
-        <v>71</v>
+        <v>106</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -792,7 +804,13 @@
         <v>1</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
+      </c>
+      <c r="F4" t="s">
+        <v>71</v>
+      </c>
+      <c r="G4" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -809,7 +827,13 @@
         <v>1</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>76</v>
+        <v>75</v>
+      </c>
+      <c r="F5" t="s">
+        <v>71</v>
+      </c>
+      <c r="G5" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -826,7 +850,13 @@
         <v>1</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
+      </c>
+      <c r="F6" t="s">
+        <v>71</v>
+      </c>
+      <c r="G6" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -843,7 +873,13 @@
         <v>1</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
+      </c>
+      <c r="F7" t="s">
+        <v>71</v>
+      </c>
+      <c r="G7" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -860,10 +896,13 @@
         <v>1</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="F8" t="s">
-        <v>9</v>
+        <v>71</v>
+      </c>
+      <c r="G8" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -880,7 +919,13 @@
         <v>1</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
+      </c>
+      <c r="F9" t="s">
+        <v>71</v>
+      </c>
+      <c r="G9" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -897,10 +942,13 @@
         <v>2</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F10" t="s">
         <v>9</v>
+      </c>
+      <c r="G10" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -908,7 +956,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C11" t="s">
         <v>8</v>
@@ -917,7 +965,13 @@
         <v>2</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
+      </c>
+      <c r="F11" t="s">
+        <v>9</v>
+      </c>
+      <c r="G11" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -925,7 +979,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C12" t="s">
         <v>8</v>
@@ -934,7 +988,13 @@
         <v>2</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
+      </c>
+      <c r="F12" t="s">
+        <v>9</v>
+      </c>
+      <c r="G12" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -951,7 +1011,13 @@
         <v>2</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
+      </c>
+      <c r="F13" t="s">
+        <v>71</v>
+      </c>
+      <c r="G13" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -968,7 +1034,13 @@
         <v>2</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
+      </c>
+      <c r="F14" t="s">
+        <v>71</v>
+      </c>
+      <c r="G14" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -985,7 +1057,13 @@
         <v>2</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
+      </c>
+      <c r="F15" t="s">
+        <v>71</v>
+      </c>
+      <c r="G15" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -1002,7 +1080,13 @@
         <v>2</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
+      </c>
+      <c r="F16" t="s">
+        <v>71</v>
+      </c>
+      <c r="G16" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -1019,13 +1103,13 @@
         <v>2</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F17" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G17" t="s">
-        <v>71</v>
+        <v>105</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -1042,7 +1126,13 @@
         <v>2</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
+      </c>
+      <c r="F18" t="s">
+        <v>71</v>
+      </c>
+      <c r="G18" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -1059,7 +1149,13 @@
         <v>2</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
+      </c>
+      <c r="F19" t="s">
+        <v>71</v>
+      </c>
+      <c r="G19" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
@@ -1076,7 +1172,13 @@
         <v>2</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
+      </c>
+      <c r="F20" t="s">
+        <v>71</v>
+      </c>
+      <c r="G20" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
@@ -1093,7 +1195,13 @@
         <v>2</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
+      </c>
+      <c r="F21" t="s">
+        <v>71</v>
+      </c>
+      <c r="G21" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
@@ -1110,7 +1218,13 @@
         <v>2</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
+      </c>
+      <c r="F22" t="s">
+        <v>71</v>
+      </c>
+      <c r="G22" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
@@ -1127,7 +1241,13 @@
         <v>2</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
+      </c>
+      <c r="F23" t="s">
+        <v>71</v>
+      </c>
+      <c r="G23" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
@@ -1144,7 +1264,13 @@
         <v>2</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
+      </c>
+      <c r="F24" t="s">
+        <v>71</v>
+      </c>
+      <c r="G24" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
@@ -1161,7 +1287,13 @@
         <v>2</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
+      </c>
+      <c r="F25" t="s">
+        <v>71</v>
+      </c>
+      <c r="G25" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
@@ -1178,7 +1310,13 @@
         <v>2</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
+      </c>
+      <c r="F26" t="s">
+        <v>71</v>
+      </c>
+      <c r="G26" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
@@ -1195,7 +1333,13 @@
         <v>2</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
+      </c>
+      <c r="F27" t="s">
+        <v>71</v>
+      </c>
+      <c r="G27" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
@@ -1212,7 +1356,13 @@
         <v>2</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
+      </c>
+      <c r="F28" t="s">
+        <v>71</v>
+      </c>
+      <c r="G28" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
@@ -1229,7 +1379,13 @@
         <v>2</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
+      </c>
+      <c r="F29" t="s">
+        <v>71</v>
+      </c>
+      <c r="G29" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
@@ -1246,7 +1402,13 @@
         <v>2</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
+      </c>
+      <c r="F30" t="s">
+        <v>71</v>
+      </c>
+      <c r="G30" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
@@ -1263,7 +1425,13 @@
         <v>2</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
+      </c>
+      <c r="F31" t="s">
+        <v>71</v>
+      </c>
+      <c r="G31" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
@@ -1280,7 +1448,13 @@
         <v>3</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
+      </c>
+      <c r="F32" t="s">
+        <v>71</v>
+      </c>
+      <c r="G32" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>